<commit_message>
fix: correct ML attribute IDs + add verified test fixture
Attribute fixes (verified via live ML API GET /categories/{id}/attributes):
- DEFROST_SYSTEM → DEFROST_TYPE (actual ML attr ID for heladeras)
- payload-builder: add WITH_FREEZER=Sí, IS_MINIBAR=No defaults for refrigerators
- payload-builder: add POWER_SUPPLY_TYPE derived from voltage field (required by MLA1577)
- attribute-defaults.ts: add DEFROST_TYPE to LIST_DEFAULTS
- appliances.ts: update refrigerator config to use DEFROST_TYPE

New fixture: tests/fixtures/ml-real-publish-final.xlsx
- 1 heladera (MLA398582) + 1 microondas (MLA1577)
- Both confirmed leaf, listing_allowed=true via live API
- All 6 required attrs covered for heladera, all 4 for microondas
- Local image filenames (uploaded to ML CDN at publish time)
- Generator: scripts/generate-verified-fixture.ts (no auth required)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/ml-real-publish-final.xlsx
+++ b/tests/fixtures/ml-real-publish-final.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Productos" sheetId="1" r:id="rId1"/>
-    <sheet name="Instrucciones" sheetId="2" r:id="rId2"/>
+    <sheet name="Verificación" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,38 +398,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:T3"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="23.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="20.83203125" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" customWidth="1"/>
-    <col min="15" max="15" width="20.83203125" customWidth="1"/>
-    <col min="16" max="16" width="20.83203125" customWidth="1"/>
-    <col min="17" max="17" width="20.83203125" customWidth="1"/>
-    <col min="18" max="18" width="23.83203125" customWidth="1"/>
-    <col min="19" max="19" width="20.83203125" customWidth="1"/>
-    <col min="20" max="20" width="20.83203125" customWidth="1"/>
-    <col min="21" max="21" width="23.83203125" customWidth="1"/>
-    <col min="22" max="22" width="20.83203125" customWidth="1"/>
-    <col min="23" max="23" width="20.83203125" customWidth="1"/>
-    <col min="24" max="24" width="23.83203125" customWidth="1"/>
-    <col min="25" max="25" width="21.83203125" customWidth="1"/>
-    <col min="26" max="26" width="27.83203125" customWidth="1"/>
-    <col min="27" max="27" width="20.83203125" customWidth="1"/>
-    <col min="28" max="28" width="20.83203125" customWidth="1"/>
-    <col min="29" max="29" width="20.83203125" customWidth="1"/>
-    <col min="30" max="30" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="24.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="24.83203125" customWidth="1"/>
+    <col min="17" max="17" width="24.83203125" customWidth="1"/>
+    <col min="18" max="18" width="24.83203125" customWidth="1"/>
+    <col min="19" max="19" width="24.83203125" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,69 +448,39 @@
         <v>stock</v>
       </c>
       <c r="I1" t="str">
-        <v>sku</v>
+        <v>color</v>
       </c>
       <c r="J1" t="str">
-        <v>color</v>
+        <v>voltaje</v>
       </c>
       <c r="K1" t="str">
-        <v>voltaje</v>
+        <v>capacidad_litros</v>
       </c>
       <c r="L1" t="str">
-        <v>capacidad_litros</v>
+        <v>capacidad_kg</v>
       </c>
       <c r="M1" t="str">
-        <v>capacidad_kg</v>
+        <v>potencia_watts</v>
       </c>
       <c r="N1" t="str">
-        <v>potencia_watts</v>
+        <v>codigo_gtin</v>
       </c>
       <c r="O1" t="str">
-        <v>tecnologia</v>
+        <v>alto_cm</v>
       </c>
       <c r="P1" t="str">
+        <v>ancho_cm</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>profundidad_cm</v>
+      </c>
+      <c r="R1" t="str">
+        <v>imagenes</v>
+      </c>
+      <c r="S1" t="str">
         <v>garantia</v>
       </c>
-      <c r="Q1" t="str">
-        <v>envio</v>
-      </c>
-      <c r="R1" t="str">
-        <v>retiro_en_persona</v>
-      </c>
-      <c r="S1" t="str">
-        <v>envio_gratis</v>
-      </c>
       <c r="T1" t="str">
-        <v>imagenes</v>
-      </c>
-      <c r="U1" t="str">
-        <v>descripcion_larga</v>
-      </c>
-      <c r="V1" t="str">
-        <v>codigo_gtin</v>
-      </c>
-      <c r="W1" t="str">
-        <v>fabricante</v>
-      </c>
-      <c r="X1" t="str">
-        <v>tipo_alimentacion</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>requiere_armado</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>incluye_manual_armado</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>alto_cm</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>ancho_cm</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>profundidad_cm</v>
-      </c>
-      <c r="AD1" t="str">
         <v>categoria_ml</v>
       </c>
     </row>
@@ -529,7 +489,7 @@
         <v>Heladera Samsung No Frost 290L Blanca</v>
       </c>
       <c r="B2" t="str">
-        <v>Heladera Samsung no frost 290 litros blanca nueva 220V garantia 12 meses modelo RT29FARADWW</v>
+        <v>heladera samsung no frost 290 litros blanca nueva con freezer inverter energía eficiente</v>
       </c>
       <c r="C2" t="str">
         <v>heladera</v>
@@ -538,82 +498,52 @@
         <v>Samsung</v>
       </c>
       <c r="E2" t="str">
-        <v>RT29FARADWW</v>
+        <v>RT29K5710S8</v>
       </c>
       <c r="F2" t="str">
-        <v>nuevo</v>
-      </c>
-      <c r="G2" t="str">
+        <v>new</v>
+      </c>
+      <c r="G2">
         <v>450000</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H2">
         <v>1</v>
       </c>
       <c r="I2" t="str">
-        <v>SAM-RT29FARADWW</v>
+        <v>Blanco</v>
       </c>
       <c r="J2" t="str">
-        <v>Blanco</v>
+        <v>220V</v>
       </c>
       <c r="K2" t="str">
-        <v>220V</v>
+        <v>290</v>
       </c>
       <c r="L2" t="str">
-        <v>290</v>
+        <v/>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>7509546069525</v>
       </c>
       <c r="O2" t="str">
-        <v>No Frost</v>
+        <v>165</v>
       </c>
       <c r="P2" t="str">
+        <v>59</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>65</v>
+      </c>
+      <c r="R2" t="str">
+        <v>heladera-frente.jpg</v>
+      </c>
+      <c r="S2" t="str">
         <v>12 meses</v>
       </c>
-      <c r="Q2" t="str">
-        <v>not_specified</v>
-      </c>
-      <c r="R2" t="str">
-        <v>si</v>
-      </c>
-      <c r="S2" t="str">
-        <v>no</v>
-      </c>
       <c r="T2" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/8/89/Refrigerator.jpg|https://upload.wikimedia.org/wikipedia/commons/b/b8/Fridge.jpg</v>
-      </c>
-      <c r="U2" t="str">
-        <v>Heladera Samsung No Frost RT29FARADWW de 290 litros. Tecnologia No Frost: elimina la escarcha automaticamente. Capacidad total: 290 litros (210L heladera + 80L freezer). Panel de control en la puerta. Alarma de puerta abierta. Iluminacion LED interior. Estantes de vidrio templado. Incluye garantia oficial Samsung de 12 meses.</v>
-      </c>
-      <c r="V2" t="str">
-        <v>7709545018831</v>
-      </c>
-      <c r="W2" t="str">
-        <v>Samsung Electronics Argentina S.A.</v>
-      </c>
-      <c r="X2" t="str">
-        <v>220V</v>
-      </c>
-      <c r="Y2" t="str">
-        <v>no</v>
-      </c>
-      <c r="Z2" t="str">
-        <v>no</v>
-      </c>
-      <c r="AA2" t="str">
-        <v>172</v>
-      </c>
-      <c r="AB2" t="str">
-        <v>60</v>
-      </c>
-      <c r="AC2" t="str">
-        <v>65</v>
-      </c>
-      <c r="AD2" t="str">
-        <v/>
+        <v>MLA398582</v>
       </c>
     </row>
     <row r="3">
@@ -621,7 +551,7 @@
         <v>Microondas Samsung 23L 1150W Blanco</v>
       </c>
       <c r="B3" t="str">
-        <v>Microondas Samsung 23 litros 1150 watts blanco nuevo 220V modelo MS23K3513AW garantia 12 meses</v>
+        <v>microondas samsung 23 litros 1150 watts blanco nuevo digital cocina</v>
       </c>
       <c r="C3" t="str">
         <v>microondas</v>
@@ -630,245 +560,258 @@
         <v>Samsung</v>
       </c>
       <c r="E3" t="str">
-        <v>MS23K3513AW</v>
+        <v>MG23K3575AW</v>
       </c>
       <c r="F3" t="str">
-        <v>nuevo</v>
-      </c>
-      <c r="G3" t="str">
-        <v>115000</v>
-      </c>
-      <c r="H3" t="str">
+        <v>new</v>
+      </c>
+      <c r="G3">
+        <v>95000</v>
+      </c>
+      <c r="H3">
         <v>1</v>
       </c>
       <c r="I3" t="str">
-        <v>SAM-MS23K3513AW</v>
+        <v>Blanco</v>
       </c>
       <c r="J3" t="str">
-        <v>Blanco</v>
+        <v>220V</v>
       </c>
       <c r="K3" t="str">
-        <v>220V</v>
+        <v>23</v>
       </c>
       <c r="L3" t="str">
-        <v>23</v>
+        <v/>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>1150</v>
       </c>
       <c r="N3" t="str">
-        <v>1150</v>
+        <v>8806092023307</v>
       </c>
       <c r="O3" t="str">
-        <v/>
+        <v>30</v>
       </c>
       <c r="P3" t="str">
+        <v>52</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>41</v>
+      </c>
+      <c r="R3" t="str">
+        <v>microondas-frente.jpg</v>
+      </c>
+      <c r="S3" t="str">
         <v>12 meses</v>
       </c>
-      <c r="Q3" t="str">
-        <v>not_specified</v>
-      </c>
-      <c r="R3" t="str">
-        <v>si</v>
-      </c>
-      <c r="S3" t="str">
-        <v>no</v>
-      </c>
       <c r="T3" t="str">
-        <v>https://placehold.co/800x600/f5f5f5/333333.jpg?text=Microondas|https://placehold.co/800x600/e8e8e8/333333.jpg?text=Microondas+interior</v>
-      </c>
-      <c r="U3" t="str">
-        <v>Microondas Samsung MS23K3513AW de 23 litros y 1150 watts. Panel de control con perillas de tiempo y potencia. 5 niveles de potencia ajustables. Funcion de descongelado automatico por peso. Plato giratorio de vidrio de 28.8 cm de diametro. Incluye garantia oficial Samsung de 12 meses.</v>
-      </c>
-      <c r="V3" t="str">
-        <v/>
-      </c>
-      <c r="W3" t="str">
-        <v>Samsung Electronics Argentina S.A.</v>
-      </c>
-      <c r="X3" t="str">
-        <v>220V</v>
-      </c>
-      <c r="Y3" t="str">
-        <v>no</v>
-      </c>
-      <c r="Z3" t="str">
-        <v>no</v>
-      </c>
-      <c r="AA3" t="str">
-        <v>27</v>
-      </c>
-      <c r="AB3" t="str">
-        <v>52</v>
-      </c>
-      <c r="AC3" t="str">
-        <v>40</v>
-      </c>
-      <c r="AD3" t="str">
-        <v/>
+        <v>MLA1577</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:C26"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>ARCHIVO DE TEST — PUBLICACION REAL EN MERCADO LIBRE</v>
+        <v>FIXTURE VERIFICATION — ml-real-publish-final.xlsx</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Generado por FastPublisher — scripts/generate-real-publish-test.ts</v>
+        <v>Generated: 2026-05-13T20:48:18.770Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Generado: 2026-05-13T16:07:39.980Z</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v/>
+        <v>Field</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Heladera</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Microondas</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>IMPORTANTE — LEER ANTES DE USAR</v>
+        <v>Product</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Heladera Samsung No Frost 290L Blanca</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Microondas Samsung 23L 1150W Blanco</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>categoria_ml</v>
+      </c>
+      <c r="B6" t="str">
+        <v>MLA398582</v>
+      </c>
+      <c r="C6" t="str">
+        <v>MLA1577</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>1. Este archivo esta disenado para pruebas de publicacion REAL en Mercado Libre.</v>
+        <v>Is leaf</v>
+      </c>
+      <c r="B7" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C7" t="str">
+        <v>YES</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2. Usar UNICAMENTE con MERCADOLIBRE_DRY_RUN=false (publicacion real activada).</v>
+        <v>listing_allowed</v>
+      </c>
+      <c r="B8" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C8" t="str">
+        <v>YES</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>3. Las imagenes fueron verificadas HTTP 200 al momento de generar este archivo.</v>
+        <v>All required attrs</v>
+      </c>
+      <c r="B9" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C9" t="str">
+        <v>YES</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>GTIN</v>
+      </c>
+      <c r="B10" t="str">
+        <v>7509546069525</v>
+      </c>
+      <c r="C10" t="str">
+        <v>8806092023307</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PRODUCTOS INCLUIDOS</v>
+        <v>Dimensions (HxWxD cm)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>165x59x65</v>
+      </c>
+      <c r="C11" t="str">
+        <v>30x52x41</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Fila</v>
+        <v>Images (local)</v>
       </c>
       <c r="B12" t="str">
-        <v>Producto</v>
+        <v>heladera-frente.jpg</v>
       </c>
       <c r="C12" t="str">
-        <v>Marca</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Categoria esperada</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Precio ARS</v>
+        <v>microondas-frente.jpg</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Heladera Samsung No Frost 290L Blanca</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Samsung</v>
-      </c>
-      <c r="D13" t="str">
-        <v>MLA-REFRIGERATORS</v>
-      </c>
-      <c r="E13" t="str">
-        <v>450.000</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>3</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Microondas Samsung 23L 1150W Blanco</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Samsung</v>
-      </c>
-      <c r="D14" t="str">
-        <v>MLA-MICROWAVES</v>
-      </c>
-      <c r="E14" t="str">
-        <v>115.000</v>
+        <v>Required attributes — Heladera (MLA398582)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>BRAND</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Samsung</v>
+      </c>
+      <c r="C15" t="str">
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>IMAGENES VERIFICADAS (HTTP 200 al generar)</v>
+        <v>MODEL</v>
+      </c>
+      <c r="B16" t="str">
+        <v>RT29K5710S8</v>
+      </c>
+      <c r="C16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Heladera img1</v>
+        <v>WITH_FREEZER</v>
       </c>
       <c r="B17" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/8/89/Refrigerator.jpg</v>
+        <v>Sí (id=242085)</v>
+      </c>
+      <c r="C17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Heladera img2</v>
+        <v>IS_MINIBAR</v>
       </c>
       <c r="B18" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/b/b8/Fridge.jpg</v>
+        <v>No (id=242084)</v>
+      </c>
+      <c r="C18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Microondas img1</v>
+        <v>DEFROST_TYPE</v>
       </c>
       <c r="B19" t="str">
-        <v>https://placehold.co/800x600/f5f5f5/333333.jpg?text=Microondas</v>
+        <v>No frost (id=2496258)</v>
+      </c>
+      <c r="C19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Microondas img2</v>
+        <v>TOTAL_CAPACITY</v>
       </c>
       <c r="B20" t="str">
-        <v>https://placehold.co/800x600/e8e8e8/333333.jpg?text=Microondas+interior</v>
+        <v>290 L</v>
+      </c>
+      <c r="C20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -878,143 +821,56 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENVIO</v>
+        <v>Required attributes — Microondas (MLA1577)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Ambos productos usan envio=not_specified (mas seguro — evita errores de me2).</v>
+        <v>BRAND</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v>Samsung</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Si el vendedor tiene me2 habilitado, cambiar a me2 en la columna "envio".</v>
+        <v>MODEL</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v>MG23K3575AW</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v>POWER_SUPPLY_TYPE</v>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v>Corriente doméstica (id=49713698)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>CATEGORIA ML (categoria_ml)</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>La columna "categoria_ml" esta vacia. El sistema la resuelve automaticamente.</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Si la resolucion automatica falla, ingresar el ID exacto de ML (ej: MLA1577).</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Recordar: ML requiere categoria HOJA (sin hijos).</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>ATRIBUTOS INCLUIDOS</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>codigo_gtin</v>
-      </c>
-      <c r="B32" t="str">
-        <v>7709545018831 (heladera) → GTIN en ML (requerido por algunas categorias)</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>fabricante</v>
-      </c>
-      <c r="B33" t="str">
-        <v>Samsung Electronics Argentina S.A. → MANUFACTURER en ML</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>tipo_alimentacion</v>
-      </c>
-      <c r="B34" t="str">
-        <v>220V → POWER_SUPPLY_TYPE en ML</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>requiere_armado</v>
-      </c>
-      <c r="B35" t="str">
-        <v>no → REQUIRES_ASSEMBLY en ML</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>alto_cm</v>
-      </c>
-      <c r="B36" t="str">
-        <v>172 (heladera) / 27 (microondas) → HEIGHT en ML</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>ancho_cm</v>
-      </c>
-      <c r="B37" t="str">
-        <v>60 (heladera) / 52 (microondas) → WIDTH en ML</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>profundidad_cm</v>
-      </c>
-      <c r="B38" t="str">
-        <v>65 (heladera) / 40 (microondas) → DEPTH en ML</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>QUE HACER SI FALLA</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>1. Revisar mlResponse en PublishHistory (panel Historial).</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>2. Causas comunes: imagenes no accesibles, categoria incorrecta, atributo faltante.</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>3. Ver docs/mercadolibre-real-publish-errors.md para referencia de errores.</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>4. Si la categoria falla: agregar ID exacto en columna "categoria_ml".</v>
+        <v>COLOR</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v>Blanco (id=52055)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>